<commit_message>
Add 26 EMBA students (114 Huanan class) to students.xlsx
Course5: 114C25502-114C25527, 5 groups from 114級華南專班

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/students.xlsx
+++ b/data/students.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E98"/>
+  <dimension ref="A1:E124"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -2072,9 +2072,451 @@
         <v>113C26531</v>
       </c>
     </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B99" t="str">
+        <v>114C25502</v>
+      </c>
+      <c r="C99" t="str">
+        <v>顏本寧</v>
+      </c>
+      <c r="D99" t="str">
+        <v/>
+      </c>
+      <c r="E99" t="str">
+        <v>114C25502</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B100" t="str">
+        <v>114C25503</v>
+      </c>
+      <c r="C100" t="str">
+        <v>羅子翔</v>
+      </c>
+      <c r="D100" t="str">
+        <v/>
+      </c>
+      <c r="E100" t="str">
+        <v>114C25503</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B101" t="str">
+        <v>114C25504</v>
+      </c>
+      <c r="C101" t="str">
+        <v>陳彥男</v>
+      </c>
+      <c r="D101" t="str">
+        <v/>
+      </c>
+      <c r="E101" t="str">
+        <v>114C25504</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B102" t="str">
+        <v>114C25505</v>
+      </c>
+      <c r="C102" t="str">
+        <v>詹富進</v>
+      </c>
+      <c r="D102" t="str">
+        <v/>
+      </c>
+      <c r="E102" t="str">
+        <v>114C25505</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B103" t="str">
+        <v>114C25506</v>
+      </c>
+      <c r="C103" t="str">
+        <v>郭靖騰</v>
+      </c>
+      <c r="D103" t="str">
+        <v/>
+      </c>
+      <c r="E103" t="str">
+        <v>114C25506</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B104" t="str">
+        <v>114C25507</v>
+      </c>
+      <c r="C104" t="str">
+        <v>葉昶緒</v>
+      </c>
+      <c r="D104" t="str">
+        <v/>
+      </c>
+      <c r="E104" t="str">
+        <v>114C25507</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B105" t="str">
+        <v>114C25508</v>
+      </c>
+      <c r="C105" t="str">
+        <v>湯凱閎</v>
+      </c>
+      <c r="D105" t="str">
+        <v/>
+      </c>
+      <c r="E105" t="str">
+        <v>114C25508</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B106" t="str">
+        <v>114C25509</v>
+      </c>
+      <c r="C106" t="str">
+        <v>謝安和</v>
+      </c>
+      <c r="D106" t="str">
+        <v/>
+      </c>
+      <c r="E106" t="str">
+        <v>114C25509</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B107" t="str">
+        <v>114C25510</v>
+      </c>
+      <c r="C107" t="str">
+        <v>余清廉</v>
+      </c>
+      <c r="D107" t="str">
+        <v/>
+      </c>
+      <c r="E107" t="str">
+        <v>114C25510</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B108" t="str">
+        <v>114C25511</v>
+      </c>
+      <c r="C108" t="str">
+        <v>洪誠聰</v>
+      </c>
+      <c r="D108" t="str">
+        <v/>
+      </c>
+      <c r="E108" t="str">
+        <v>114C25511</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B109" t="str">
+        <v>114C25512</v>
+      </c>
+      <c r="C109" t="str">
+        <v>湯顯智</v>
+      </c>
+      <c r="D109" t="str">
+        <v/>
+      </c>
+      <c r="E109" t="str">
+        <v>114C25512</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B110" t="str">
+        <v>114C25513</v>
+      </c>
+      <c r="C110" t="str">
+        <v>林明毅</v>
+      </c>
+      <c r="D110" t="str">
+        <v/>
+      </c>
+      <c r="E110" t="str">
+        <v>114C25513</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B111" t="str">
+        <v>114C25514</v>
+      </c>
+      <c r="C111" t="str">
+        <v>林長青</v>
+      </c>
+      <c r="D111" t="str">
+        <v/>
+      </c>
+      <c r="E111" t="str">
+        <v>114C25514</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B112" t="str">
+        <v>114C25515</v>
+      </c>
+      <c r="C112" t="str">
+        <v>吳佳惠</v>
+      </c>
+      <c r="D112" t="str">
+        <v/>
+      </c>
+      <c r="E112" t="str">
+        <v>114C25515</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B113" t="str">
+        <v>114C25516</v>
+      </c>
+      <c r="C113" t="str">
+        <v>林美蘭</v>
+      </c>
+      <c r="D113" t="str">
+        <v/>
+      </c>
+      <c r="E113" t="str">
+        <v>114C25516</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B114" t="str">
+        <v>114C25517</v>
+      </c>
+      <c r="C114" t="str">
+        <v>賴家駿</v>
+      </c>
+      <c r="D114" t="str">
+        <v/>
+      </c>
+      <c r="E114" t="str">
+        <v>114C25517</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B115" t="str">
+        <v>114C25518</v>
+      </c>
+      <c r="C115" t="str">
+        <v>廖清宏</v>
+      </c>
+      <c r="D115" t="str">
+        <v/>
+      </c>
+      <c r="E115" t="str">
+        <v>114C25518</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B116" t="str">
+        <v>114C25519</v>
+      </c>
+      <c r="C116" t="str">
+        <v>葉智文</v>
+      </c>
+      <c r="D116" t="str">
+        <v/>
+      </c>
+      <c r="E116" t="str">
+        <v>114C25519</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B117" t="str">
+        <v>114C25520</v>
+      </c>
+      <c r="C117" t="str">
+        <v>黃國華</v>
+      </c>
+      <c r="D117" t="str">
+        <v/>
+      </c>
+      <c r="E117" t="str">
+        <v>114C25520</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B118" t="str">
+        <v>114C25521</v>
+      </c>
+      <c r="C118" t="str">
+        <v>張藝齡</v>
+      </c>
+      <c r="D118" t="str">
+        <v/>
+      </c>
+      <c r="E118" t="str">
+        <v>114C25521</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B119" t="str">
+        <v>114C25522</v>
+      </c>
+      <c r="C119" t="str">
+        <v>陳堯麟</v>
+      </c>
+      <c r="D119" t="str">
+        <v/>
+      </c>
+      <c r="E119" t="str">
+        <v>114C25522</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B120" t="str">
+        <v>114C25523</v>
+      </c>
+      <c r="C120" t="str">
+        <v>卜竹如</v>
+      </c>
+      <c r="D120" t="str">
+        <v/>
+      </c>
+      <c r="E120" t="str">
+        <v>114C25523</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B121" t="str">
+        <v>114C25524</v>
+      </c>
+      <c r="C121" t="str">
+        <v>黃宣瑋</v>
+      </c>
+      <c r="D121" t="str">
+        <v/>
+      </c>
+      <c r="E121" t="str">
+        <v>114C25524</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B122" t="str">
+        <v>114C25525</v>
+      </c>
+      <c r="C122" t="str">
+        <v>呂軍林</v>
+      </c>
+      <c r="D122" t="str">
+        <v/>
+      </c>
+      <c r="E122" t="str">
+        <v>114C25525</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B123" t="str">
+        <v>114C25526</v>
+      </c>
+      <c r="C123" t="str">
+        <v>張亦良</v>
+      </c>
+      <c r="D123" t="str">
+        <v/>
+      </c>
+      <c r="E123" t="str">
+        <v>114C25526</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B124" t="str">
+        <v>114C25527</v>
+      </c>
+      <c r="C124" t="str">
+        <v>張馥麟</v>
+      </c>
+      <c r="D124" t="str">
+        <v/>
+      </c>
+      <c r="E124" t="str">
+        <v>114C25527</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E98"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E124"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 53 course6 (115-1 程式語言) students to roster
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/students.xlsx
+++ b/data/students.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E101"/>
+  <dimension ref="A1:E154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18.83203125" customWidth="1" min="1" max="1"/>
@@ -2148,7 +2148,6 @@
           <t>黃聖傑</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr"/>
       <c r="E77" t="inlineStr">
         <is>
           <t>112370231</t>
@@ -2171,7 +2170,6 @@
           <t>徐之晨</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr"/>
       <c r="E78" t="inlineStr">
         <is>
           <t>112370121</t>
@@ -2194,7 +2192,6 @@
           <t>江英豪</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr"/>
       <c r="E79" t="inlineStr">
         <is>
           <t>115378003</t>
@@ -2217,7 +2214,6 @@
           <t>蔡承祐</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr"/>
       <c r="E80" t="inlineStr">
         <is>
           <t>115378010</t>
@@ -2240,7 +2236,6 @@
           <t>蘇鈺涵</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr"/>
       <c r="E81" t="inlineStr">
         <is>
           <t>115378015</t>
@@ -2263,7 +2258,6 @@
           <t>冉云豪</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr"/>
       <c r="E82" t="inlineStr">
         <is>
           <t>115378016</t>
@@ -2286,7 +2280,6 @@
           <t>吳楷涵</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr"/>
       <c r="E83" t="inlineStr">
         <is>
           <t>115378017</t>
@@ -2309,7 +2302,6 @@
           <t>張晏婷</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr"/>
       <c r="E84" t="inlineStr">
         <is>
           <t>115378023</t>
@@ -2332,7 +2324,6 @@
           <t>紀佑威</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr"/>
       <c r="E85" t="inlineStr">
         <is>
           <t>115378036</t>
@@ -2355,7 +2346,6 @@
           <t>劉主平</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr"/>
       <c r="E86" t="inlineStr">
         <is>
           <t>115378044</t>
@@ -2378,7 +2368,6 @@
           <t>王浩宇</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr"/>
       <c r="E87" t="inlineStr">
         <is>
           <t>115378049</t>
@@ -2401,7 +2390,6 @@
           <t>柯家恩</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr"/>
       <c r="E88" t="inlineStr">
         <is>
           <t>115378054</t>
@@ -2424,7 +2412,6 @@
           <t>曾旭辰</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr"/>
       <c r="E89" t="inlineStr">
         <is>
           <t>115378056</t>
@@ -2447,7 +2434,6 @@
           <t>陳冠豪</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr"/>
       <c r="E90" t="inlineStr">
         <is>
           <t>115378061</t>
@@ -2470,7 +2456,6 @@
           <t>簡祺倫</t>
         </is>
       </c>
-      <c r="D91" t="inlineStr"/>
       <c r="E91" t="inlineStr">
         <is>
           <t>115378062</t>
@@ -2493,7 +2478,6 @@
           <t>陳俊曄</t>
         </is>
       </c>
-      <c r="D92" t="inlineStr"/>
       <c r="E92" t="inlineStr">
         <is>
           <t>115378065</t>
@@ -2516,7 +2500,6 @@
           <t>翁郁</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr"/>
       <c r="E93" t="inlineStr">
         <is>
           <t>115378069</t>
@@ -2539,7 +2522,6 @@
           <t>謝孟峰</t>
         </is>
       </c>
-      <c r="D94" t="inlineStr"/>
       <c r="E94" t="inlineStr">
         <is>
           <t>115378070</t>
@@ -2562,7 +2544,6 @@
           <t>林楷融</t>
         </is>
       </c>
-      <c r="D95" t="inlineStr"/>
       <c r="E95" t="inlineStr">
         <is>
           <t>115378076</t>
@@ -2585,7 +2566,6 @@
           <t>陳奕承</t>
         </is>
       </c>
-      <c r="D96" t="inlineStr"/>
       <c r="E96" t="inlineStr">
         <is>
           <t>114378024</t>
@@ -2608,7 +2588,6 @@
           <t>楊佳芯</t>
         </is>
       </c>
-      <c r="D97" t="inlineStr"/>
       <c r="E97" t="inlineStr">
         <is>
           <t>114378082</t>
@@ -2631,7 +2610,6 @@
           <t>劉家蓁</t>
         </is>
       </c>
-      <c r="D98" t="inlineStr"/>
       <c r="E98" t="inlineStr">
         <is>
           <t>114378084</t>
@@ -2654,7 +2632,6 @@
           <t>高耘謙</t>
         </is>
       </c>
-      <c r="D99" t="inlineStr"/>
       <c r="E99" t="inlineStr">
         <is>
           <t>114578011</t>
@@ -2677,7 +2654,6 @@
           <t>李雨蓁</t>
         </is>
       </c>
-      <c r="D100" t="inlineStr"/>
       <c r="E100" t="inlineStr">
         <is>
           <t>114578021</t>
@@ -2700,10 +2676,1228 @@
           <t>吳俊翊</t>
         </is>
       </c>
-      <c r="D101" t="inlineStr"/>
       <c r="E101" t="inlineStr">
         <is>
           <t>114578032</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>114370104</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>吳欣桐</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr"/>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>114370104</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>114370109</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>蘇宥慈</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr"/>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>114370109</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>115370101</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>何維榛</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr"/>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>115370101</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>115370102</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>邱慈閑</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr"/>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>115370102</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>115370103</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>廖宏恩</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr"/>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>115370103</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>115370104</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>施皓勛</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr"/>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>115370104</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>115370105</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>李培瑤</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr"/>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>115370105</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>115370106</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>江俊緯</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr"/>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>115370106</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>115370108</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>陳宥安</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr"/>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>115370108</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>115370109</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>陳宥叡</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr"/>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>115370109</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>115370110</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>王彥清</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr"/>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>115370110</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>115370111</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>廖浚淇</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr"/>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>115370111</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>115370112</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>吳亞叡</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr"/>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>115370112</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>115370113</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>張洧豪</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr"/>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>115370113</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>115370114</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>陸捷</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr"/>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>115370114</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>115370115</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>蔡幸恩</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr"/>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>115370115</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>115370116</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>康博閎</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr"/>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>115370116</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>115370117</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>莫家葳</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr"/>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>115370117</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>115370118</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>王義翔</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr"/>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>115370118</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>115370119</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>譚佑捷</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr"/>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>115370119</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>115370120</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>林子佑</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr"/>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>115370120</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>115370121</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>陳右珊</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr"/>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>115370121</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>115370122</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>楊仁佑</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr"/>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>115370122</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>115370123</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>林洋宇</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr"/>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>115370123</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>115370124</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>蔡承諺</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr"/>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>115370124</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>115370125</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>蘇振綸</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr"/>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>115370125</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>115370126</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>陳億承</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr"/>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>115370126</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>115370127</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>沈奕瑱</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr"/>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>115370127</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>115370128</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>翁敏瑄</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr"/>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>115370128</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>115370129</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>傅可喬</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr"/>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>115370129</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>115370130</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>易品妘</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr"/>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>115370130</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>115370131</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>張薇婷</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr"/>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>115370131</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>115370132</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>蕭志杰</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr"/>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>115370132</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>115370133</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>彭榆真</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr"/>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>115370133</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>115370134</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>鄧妤溱</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr"/>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>115370134</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>115370135</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>蔡其叡</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr"/>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>115370135</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>115370136</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>翁翊宸</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr"/>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>115370136</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>115370137</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>陳柏霖</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr"/>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>115370137</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>115370138</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>蔡侑霖</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr"/>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>115370138</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>115370139</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>許凡羿</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr"/>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>115370139</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>115370140</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>宋世瑞</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr"/>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>115370140</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>115370141</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>張瑞晏</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr"/>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>115370141</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>115370142</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>賴妍馨</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr"/>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>115370142</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>115370143</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>馮志恭</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr"/>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>115370143</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>115370144</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>謝玉玄</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr"/>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>115370144</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>115370145</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>曾千財</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr"/>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>115370145</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>115370146</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>歐水愛</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr"/>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>115370146</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>115370147</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>思益邦</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr"/>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>115370147</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>115370148</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>楊詠訊</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr"/>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>115370148</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>112370116</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>吳冠谷</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr"/>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>112370116</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>112370138</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>施皓偉</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr"/>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>112370138</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>112370140</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>施廷儒</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr"/>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>112370140</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>course6</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>112540024</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>廖芷葶</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr"/>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>112540024</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove course1 (機器視覺) students from roster
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/students.xlsx
+++ b/data/students.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E154"/>
+  <dimension ref="A1:E135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18.83203125" customWidth="1" min="1" max="1"/>
@@ -485,418 +485,418 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>course1</t>
+          <t>course5</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>113378004</t>
+          <t>113C26501</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>蔡孟紘</t>
+          <t>蔡彰哲</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>113378004</t>
+          <t>113C26501</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>course1</t>
+          <t>course5</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>113378082</t>
+          <t>113C26502</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>徐碩襄</t>
+          <t>朱文怡</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>113378082</t>
+          <t>113C26502</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>course1</t>
+          <t>course5</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>113378083</t>
+          <t>113C26503</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>朱翊瑄</t>
+          <t>王光輝</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>113378083</t>
+          <t>113C26503</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>course1</t>
+          <t>course5</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>114378006</t>
+          <t>113C26504</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>周冠瑋</t>
+          <t>江明憲</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>114378006</t>
+          <t>113C26504</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>course1</t>
+          <t>course5</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>114378008</t>
+          <t>113C26505</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>王柏翔</t>
+          <t>徐詩琴</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>114378008</t>
+          <t>113C26505</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>course1</t>
+          <t>course5</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>114378019</t>
+          <t>113C26506</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>鄧雅馨</t>
+          <t>唐青文</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>114378019</t>
+          <t>113C26506</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>course1</t>
+          <t>course5</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>114378025</t>
+          <t>113C26507</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>鄭怡仙</t>
+          <t>鄭昱暘</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>114378025</t>
+          <t>113C26507</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>course1</t>
+          <t>course5</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>114378028</t>
+          <t>113C26508</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>范辰瑋</t>
+          <t>曾任健</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>114378028</t>
+          <t>113C26508</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>course1</t>
+          <t>course5</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>114378033</t>
+          <t>113C26509</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>蘇煒傑</t>
+          <t>鄧宇翔</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>114378033</t>
+          <t>113C26509</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>course1</t>
+          <t>course5</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>114378036</t>
+          <t>113C26511</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>廖晨宇</t>
+          <t>許志鴻</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>114378036</t>
+          <t>113C26511</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>course1</t>
+          <t>course5</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>114378042</t>
+          <t>113C26512</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>李彤</t>
+          <t>陳佩宜</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>114378042</t>
+          <t>113C26512</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>course1</t>
+          <t>course5</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>114378048</t>
+          <t>113C26513</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>吳鎵全</t>
+          <t>廖倫群</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>114378048</t>
+          <t>113C26513</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>course1</t>
+          <t>course5</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>114378056</t>
+          <t>113C26514</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>莊以謙</t>
+          <t>李後熙</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>114378056</t>
+          <t>113C26514</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>course1</t>
+          <t>course5</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>114378058</t>
+          <t>113C26515</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>李亭萱</t>
+          <t>曾榮富</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>114378058</t>
+          <t>113C26515</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>course1</t>
+          <t>course5</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>114378061</t>
+          <t>113C26516</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>段瑞城</t>
+          <t>巫大宇</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>114378061</t>
+          <t>113C26516</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>course1</t>
+          <t>course5</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>114378071</t>
+          <t>113C26517</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>蔡佳妤</t>
+          <t>劉永霖</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>114378071</t>
+          <t>113C26517</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>course1</t>
+          <t>course5</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>114378075</t>
+          <t>113C26518</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>鄭宜諠</t>
+          <t>顧國立</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>114378075</t>
+          <t>113C26518</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>course1</t>
+          <t>course5</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>114378079</t>
+          <t>113C26519</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>馮宣穎</t>
+          <t>盧仁傑</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>114378079</t>
+          <t>113C26519</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>course1</t>
+          <t>course5</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>114378084</t>
+          <t>113C26520</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>劉家蓁</t>
+          <t>魏明照</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>114378084</t>
+          <t>113C26520</t>
         </is>
       </c>
     </row>
@@ -908,17 +908,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>113C26501</t>
+          <t>113C26521</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>蔡彰哲</t>
+          <t>陳勇廷</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>113C26501</t>
+          <t>113C26521</t>
         </is>
       </c>
     </row>
@@ -930,17 +930,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>113C26502</t>
+          <t>113C26522</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>朱文怡</t>
+          <t>陳麗玲</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>113C26502</t>
+          <t>113C26522</t>
         </is>
       </c>
     </row>
@@ -952,17 +952,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>113C26503</t>
+          <t>113C26523</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>王光輝</t>
+          <t>楊光倫</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>113C26503</t>
+          <t>113C26523</t>
         </is>
       </c>
     </row>
@@ -974,17 +974,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>113C26504</t>
+          <t>113C26524</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>江明憲</t>
+          <t>黃乙民</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>113C26504</t>
+          <t>113C26524</t>
         </is>
       </c>
     </row>
@@ -996,17 +996,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>113C26505</t>
+          <t>113C26525</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>徐詩琴</t>
+          <t>姚昶志</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>113C26505</t>
+          <t>113C26525</t>
         </is>
       </c>
     </row>
@@ -1018,17 +1018,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>113C26506</t>
+          <t>113C26526</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>唐青文</t>
+          <t>張瑋祥</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>113C26506</t>
+          <t>113C26526</t>
         </is>
       </c>
     </row>
@@ -1040,17 +1040,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>113C26507</t>
+          <t>113C26527</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>鄭昱暘</t>
+          <t>李菀頻</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>113C26507</t>
+          <t>113C26527</t>
         </is>
       </c>
     </row>
@@ -1062,17 +1062,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>113C26508</t>
+          <t>113C26528</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>曾任健</t>
+          <t>陳穎婕</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>113C26508</t>
+          <t>113C26528</t>
         </is>
       </c>
     </row>
@@ -1084,17 +1084,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>113C26509</t>
+          <t>113C26529</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>鄧宇翔</t>
+          <t>許育銘</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>113C26509</t>
+          <t>113C26529</t>
         </is>
       </c>
     </row>
@@ -1106,17 +1106,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>113C26511</t>
+          <t>113C26530</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>許志鴻</t>
+          <t>王子欣</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>113C26511</t>
+          <t>113C26530</t>
         </is>
       </c>
     </row>
@@ -1128,17 +1128,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>113C26512</t>
+          <t>113C26531</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>陳佩宜</t>
+          <t>邱明加</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>113C26512</t>
+          <t>113C26531</t>
         </is>
       </c>
     </row>
@@ -1150,17 +1150,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>113C26513</t>
+          <t>114C25502</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>廖倫群</t>
+          <t>顏本寧</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>113C26513</t>
+          <t>114C25502</t>
         </is>
       </c>
     </row>
@@ -1172,17 +1172,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>113C26514</t>
+          <t>114C25503</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>李後熙</t>
+          <t>羅子翔</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>113C26514</t>
+          <t>114C25503</t>
         </is>
       </c>
     </row>
@@ -1194,17 +1194,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>113C26515</t>
+          <t>114C25504</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>曾榮富</t>
+          <t>陳彥男</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>113C26515</t>
+          <t>114C25504</t>
         </is>
       </c>
     </row>
@@ -1216,17 +1216,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>113C26516</t>
+          <t>114C25505</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>巫大宇</t>
+          <t>詹富進</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>113C26516</t>
+          <t>114C25505</t>
         </is>
       </c>
     </row>
@@ -1238,17 +1238,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>113C26517</t>
+          <t>114C25506</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>劉永霖</t>
+          <t>郭靖騰</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>113C26517</t>
+          <t>114C25506</t>
         </is>
       </c>
     </row>
@@ -1260,17 +1260,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>113C26518</t>
+          <t>114C25507</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>顧國立</t>
+          <t>葉昶緒</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>113C26518</t>
+          <t>114C25507</t>
         </is>
       </c>
     </row>
@@ -1282,17 +1282,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>113C26519</t>
+          <t>114C25508</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>盧仁傑</t>
+          <t>湯凱閎</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>113C26519</t>
+          <t>114C25508</t>
         </is>
       </c>
     </row>
@@ -1304,17 +1304,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>113C26520</t>
+          <t>114C25509</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>魏明照</t>
+          <t>謝安和</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>113C26520</t>
+          <t>114C25509</t>
         </is>
       </c>
     </row>
@@ -1326,17 +1326,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>113C26521</t>
+          <t>114C25510</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>陳勇廷</t>
+          <t>余清廉</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>113C26521</t>
+          <t>114C25510</t>
         </is>
       </c>
     </row>
@@ -1348,17 +1348,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>113C26522</t>
+          <t>114C25511</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>陳麗玲</t>
+          <t>洪誠聰</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>113C26522</t>
+          <t>114C25511</t>
         </is>
       </c>
     </row>
@@ -1370,17 +1370,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>113C26523</t>
+          <t>114C25512</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>楊光倫</t>
+          <t>湯顯智</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>113C26523</t>
+          <t>114C25512</t>
         </is>
       </c>
     </row>
@@ -1392,17 +1392,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>113C26524</t>
+          <t>114C25513</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>黃乙民</t>
+          <t>林明毅</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>113C26524</t>
+          <t>114C25513</t>
         </is>
       </c>
     </row>
@@ -1414,17 +1414,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>113C26525</t>
+          <t>114C25514</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>姚昶志</t>
+          <t>林長青</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>113C26525</t>
+          <t>114C25514</t>
         </is>
       </c>
     </row>
@@ -1436,17 +1436,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>113C26526</t>
+          <t>114C25515</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>張瑋祥</t>
+          <t>吳佳惠</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>113C26526</t>
+          <t>114C25515</t>
         </is>
       </c>
     </row>
@@ -1458,17 +1458,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>113C26527</t>
+          <t>114C25516</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>李菀頻</t>
+          <t>林美蘭</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>113C26527</t>
+          <t>114C25516</t>
         </is>
       </c>
     </row>
@@ -1480,17 +1480,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>113C26528</t>
+          <t>114C25517</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>陳穎婕</t>
+          <t>賴家駿</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>113C26528</t>
+          <t>114C25517</t>
         </is>
       </c>
     </row>
@@ -1502,17 +1502,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>113C26529</t>
+          <t>114C25518</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>許育銘</t>
+          <t>廖清宏</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>113C26529</t>
+          <t>114C25518</t>
         </is>
       </c>
     </row>
@@ -1524,17 +1524,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>113C26530</t>
+          <t>114C25519</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>王子欣</t>
+          <t>葉智文</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>113C26530</t>
+          <t>114C25519</t>
         </is>
       </c>
     </row>
@@ -1546,17 +1546,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>113C26531</t>
+          <t>114C25520</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>邱明加</t>
+          <t>黃國華</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>113C26531</t>
+          <t>114C25520</t>
         </is>
       </c>
     </row>
@@ -1568,17 +1568,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>114C25502</t>
+          <t>114C25521</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>顏本寧</t>
+          <t>張藝齡</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>114C25502</t>
+          <t>114C25521</t>
         </is>
       </c>
     </row>
@@ -1590,17 +1590,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>114C25503</t>
+          <t>114C25522</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>羅子翔</t>
+          <t>陳堯麟</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>114C25503</t>
+          <t>114C25522</t>
         </is>
       </c>
     </row>
@@ -1612,17 +1612,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>114C25504</t>
+          <t>114C25523</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>陳彥男</t>
+          <t>卜竹如</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>114C25504</t>
+          <t>114C25523</t>
         </is>
       </c>
     </row>
@@ -1634,17 +1634,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>114C25505</t>
+          <t>114C25524</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>詹富進</t>
+          <t>黃宣瑋</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>114C25505</t>
+          <t>114C25524</t>
         </is>
       </c>
     </row>
@@ -1656,17 +1656,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>114C25506</t>
+          <t>114C25525</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>郭靖騰</t>
+          <t>呂軍林</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>114C25506</t>
+          <t>114C25525</t>
         </is>
       </c>
     </row>
@@ -1678,17 +1678,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>114C25507</t>
+          <t>114C25526</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>葉昶緒</t>
+          <t>張亦良</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>114C25507</t>
+          <t>114C25526</t>
         </is>
       </c>
     </row>
@@ -1700,435 +1700,435 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>114C25508</t>
+          <t>114C25527</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>湯凱閎</t>
+          <t>張馥麟</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>114C25508</t>
+          <t>114C25527</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>course5</t>
+          <t>course3</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>114C25509</t>
+          <t>112370231</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>謝安和</t>
+          <t>黃聖傑</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>114C25509</t>
+          <t>112370231</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>course5</t>
+          <t>course3</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>114C25510</t>
+          <t>112370121</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>余清廉</t>
+          <t>徐之晨</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>114C25510</t>
+          <t>112370121</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>course5</t>
+          <t>course3</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>114C25511</t>
+          <t>115378003</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>洪誠聰</t>
+          <t>江英豪</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>114C25511</t>
+          <t>115378003</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>course5</t>
+          <t>course3</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>114C25512</t>
+          <t>115378010</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>湯顯智</t>
+          <t>蔡承祐</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>114C25512</t>
+          <t>115378010</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>course5</t>
+          <t>course3</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>114C25513</t>
+          <t>115378015</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>林明毅</t>
+          <t>蘇鈺涵</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>114C25513</t>
+          <t>115378015</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>course5</t>
+          <t>course3</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>114C25514</t>
+          <t>115378016</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>林長青</t>
+          <t>冉云豪</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>114C25514</t>
+          <t>115378016</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>course5</t>
+          <t>course3</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>114C25515</t>
+          <t>115378017</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>吳佳惠</t>
+          <t>吳楷涵</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>114C25515</t>
+          <t>115378017</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>course5</t>
+          <t>course3</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>114C25516</t>
+          <t>115378023</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>林美蘭</t>
+          <t>張晏婷</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>114C25516</t>
+          <t>115378023</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>course5</t>
+          <t>course3</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>114C25517</t>
+          <t>115378036</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>賴家駿</t>
+          <t>紀佑威</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>114C25517</t>
+          <t>115378036</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>course5</t>
+          <t>course3</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>114C25518</t>
+          <t>115378044</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>廖清宏</t>
+          <t>劉主平</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>114C25518</t>
+          <t>115378044</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>course5</t>
+          <t>course3</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>114C25519</t>
+          <t>115378049</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>葉智文</t>
+          <t>王浩宇</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>114C25519</t>
+          <t>115378049</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>course5</t>
+          <t>course3</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>114C25520</t>
+          <t>115378054</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>黃國華</t>
+          <t>柯家恩</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>114C25520</t>
+          <t>115378054</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>course5</t>
+          <t>course3</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>114C25521</t>
+          <t>115378056</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>張藝齡</t>
+          <t>曾旭辰</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>114C25521</t>
+          <t>115378056</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>course5</t>
+          <t>course3</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>114C25522</t>
+          <t>115378061</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>陳堯麟</t>
+          <t>陳冠豪</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>114C25522</t>
+          <t>115378061</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>course5</t>
+          <t>course3</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>114C25523</t>
+          <t>115378062</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>卜竹如</t>
+          <t>簡祺倫</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>114C25523</t>
+          <t>115378062</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>course5</t>
+          <t>course3</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>114C25524</t>
+          <t>115378065</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>黃宣瑋</t>
+          <t>陳俊曄</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>114C25524</t>
+          <t>115378065</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>course5</t>
+          <t>course3</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>114C25525</t>
+          <t>115378069</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>呂軍林</t>
+          <t>翁郁</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>114C25525</t>
+          <t>115378069</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>course5</t>
+          <t>course3</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>114C25526</t>
+          <t>115378070</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>張亦良</t>
+          <t>謝孟峰</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>114C25526</t>
+          <t>115378070</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>course5</t>
+          <t>course3</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>114C25527</t>
+          <t>115378076</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>張馥麟</t>
+          <t>林楷融</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>114C25527</t>
+          <t>115378076</t>
         </is>
       </c>
     </row>
@@ -2140,17 +2140,17 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>112370231</t>
+          <t>114378024</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>黃聖傑</t>
+          <t>陳奕承</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>112370231</t>
+          <t>114378024</t>
         </is>
       </c>
     </row>
@@ -2162,17 +2162,17 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>112370121</t>
+          <t>114378082</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>徐之晨</t>
+          <t>楊佳芯</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>112370121</t>
+          <t>114378082</t>
         </is>
       </c>
     </row>
@@ -2184,17 +2184,17 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>115378003</t>
+          <t>114378084</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>江英豪</t>
+          <t>劉家蓁</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>115378003</t>
+          <t>114378084</t>
         </is>
       </c>
     </row>
@@ -2206,17 +2206,17 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>115378010</t>
+          <t>114578011</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>蔡承祐</t>
+          <t>高耘謙</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>115378010</t>
+          <t>114578011</t>
         </is>
       </c>
     </row>
@@ -2228,17 +2228,17 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>115378015</t>
+          <t>114578021</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>蘇鈺涵</t>
+          <t>李雨蓁</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>115378015</t>
+          <t>114578021</t>
         </is>
       </c>
     </row>
@@ -2250,435 +2250,435 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>115378016</t>
+          <t>114578032</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>冉云豪</t>
+          <t>吳俊翊</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>115378016</t>
+          <t>114578032</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>course3</t>
+          <t>course6</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>115378017</t>
+          <t>114370104</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>吳楷涵</t>
+          <t>吳欣桐</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>115378017</t>
+          <t>114370104</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>course3</t>
+          <t>course6</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>115378023</t>
+          <t>114370109</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>張晏婷</t>
+          <t>蘇宥慈</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>115378023</t>
+          <t>114370109</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>course3</t>
+          <t>course6</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>115378036</t>
+          <t>115370101</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>紀佑威</t>
+          <t>何維榛</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>115378036</t>
+          <t>115370101</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>course3</t>
+          <t>course6</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>115378044</t>
+          <t>115370102</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>劉主平</t>
+          <t>邱慈閑</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>115378044</t>
+          <t>115370102</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>course3</t>
+          <t>course6</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>115378049</t>
+          <t>115370103</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>王浩宇</t>
+          <t>廖宏恩</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>115378049</t>
+          <t>115370103</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>course3</t>
+          <t>course6</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>115378054</t>
+          <t>115370104</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>柯家恩</t>
+          <t>施皓勛</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>115378054</t>
+          <t>115370104</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>course3</t>
+          <t>course6</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>115378056</t>
+          <t>115370105</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>曾旭辰</t>
+          <t>李培瑤</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>115378056</t>
+          <t>115370105</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>course3</t>
+          <t>course6</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>115378061</t>
+          <t>115370106</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>陳冠豪</t>
+          <t>江俊緯</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>115378061</t>
+          <t>115370106</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>course3</t>
+          <t>course6</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>115378062</t>
+          <t>115370108</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>簡祺倫</t>
+          <t>陳宥安</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>115378062</t>
+          <t>115370108</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>course3</t>
+          <t>course6</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>115378065</t>
+          <t>115370109</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>陳俊曄</t>
+          <t>陳宥叡</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>115378065</t>
+          <t>115370109</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>course3</t>
+          <t>course6</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>115378069</t>
+          <t>115370110</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>翁郁</t>
+          <t>王彥清</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>115378069</t>
+          <t>115370110</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>course3</t>
+          <t>course6</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>115378070</t>
+          <t>115370111</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>謝孟峰</t>
+          <t>廖浚淇</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>115378070</t>
+          <t>115370111</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>course3</t>
+          <t>course6</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>115378076</t>
+          <t>115370112</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>林楷融</t>
+          <t>吳亞叡</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>115378076</t>
+          <t>115370112</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>course3</t>
+          <t>course6</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>114378024</t>
+          <t>115370113</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>陳奕承</t>
+          <t>張洧豪</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>114378024</t>
+          <t>115370113</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>course3</t>
+          <t>course6</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>114378082</t>
+          <t>115370114</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>楊佳芯</t>
+          <t>陸捷</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>114378082</t>
+          <t>115370114</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>course3</t>
+          <t>course6</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>114378084</t>
+          <t>115370115</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>劉家蓁</t>
+          <t>蔡幸恩</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>114378084</t>
+          <t>115370115</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>course3</t>
+          <t>course6</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>114578011</t>
+          <t>115370116</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>高耘謙</t>
+          <t>康博閎</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>114578011</t>
+          <t>115370116</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>course3</t>
+          <t>course6</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>114578021</t>
+          <t>115370117</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>李雨蓁</t>
+          <t>莫家葳</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>114578021</t>
+          <t>115370117</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>course3</t>
+          <t>course6</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>114578032</t>
+          <t>115370118</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>吳俊翊</t>
+          <t>王義翔</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>114578032</t>
+          <t>115370118</t>
         </is>
       </c>
     </row>
@@ -2690,18 +2690,17 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>114370104</t>
+          <t>115370119</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>吳欣桐</t>
-        </is>
-      </c>
-      <c r="D102" t="inlineStr"/>
+          <t>譚佑捷</t>
+        </is>
+      </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>114370104</t>
+          <t>115370119</t>
         </is>
       </c>
     </row>
@@ -2713,18 +2712,17 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>114370109</t>
+          <t>115370120</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>蘇宥慈</t>
-        </is>
-      </c>
-      <c r="D103" t="inlineStr"/>
+          <t>林子佑</t>
+        </is>
+      </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>114370109</t>
+          <t>115370120</t>
         </is>
       </c>
     </row>
@@ -2736,18 +2734,17 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>115370101</t>
+          <t>115370121</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>何維榛</t>
-        </is>
-      </c>
-      <c r="D104" t="inlineStr"/>
+          <t>陳右珊</t>
+        </is>
+      </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>115370101</t>
+          <t>115370121</t>
         </is>
       </c>
     </row>
@@ -2759,18 +2756,17 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>115370102</t>
+          <t>115370122</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>邱慈閑</t>
-        </is>
-      </c>
-      <c r="D105" t="inlineStr"/>
+          <t>楊仁佑</t>
+        </is>
+      </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>115370102</t>
+          <t>115370122</t>
         </is>
       </c>
     </row>
@@ -2782,18 +2778,17 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>115370103</t>
+          <t>115370123</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>廖宏恩</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr"/>
+          <t>林洋宇</t>
+        </is>
+      </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>115370103</t>
+          <t>115370123</t>
         </is>
       </c>
     </row>
@@ -2805,18 +2800,17 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>115370104</t>
+          <t>115370124</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>施皓勛</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr"/>
+          <t>蔡承諺</t>
+        </is>
+      </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>115370104</t>
+          <t>115370124</t>
         </is>
       </c>
     </row>
@@ -2828,18 +2822,17 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>115370105</t>
+          <t>115370125</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>李培瑤</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr"/>
+          <t>蘇振綸</t>
+        </is>
+      </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>115370105</t>
+          <t>115370125</t>
         </is>
       </c>
     </row>
@@ -2851,18 +2844,17 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>115370106</t>
+          <t>115370126</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>江俊緯</t>
-        </is>
-      </c>
-      <c r="D109" t="inlineStr"/>
+          <t>陳億承</t>
+        </is>
+      </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>115370106</t>
+          <t>115370126</t>
         </is>
       </c>
     </row>
@@ -2874,18 +2866,17 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>115370108</t>
+          <t>115370127</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>陳宥安</t>
-        </is>
-      </c>
-      <c r="D110" t="inlineStr"/>
+          <t>沈奕瑱</t>
+        </is>
+      </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>115370108</t>
+          <t>115370127</t>
         </is>
       </c>
     </row>
@@ -2897,18 +2888,17 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>115370109</t>
+          <t>115370128</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>陳宥叡</t>
-        </is>
-      </c>
-      <c r="D111" t="inlineStr"/>
+          <t>翁敏瑄</t>
+        </is>
+      </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>115370109</t>
+          <t>115370128</t>
         </is>
       </c>
     </row>
@@ -2920,18 +2910,17 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>115370110</t>
+          <t>115370129</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>王彥清</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr"/>
+          <t>傅可喬</t>
+        </is>
+      </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>115370110</t>
+          <t>115370129</t>
         </is>
       </c>
     </row>
@@ -2943,18 +2932,17 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>115370111</t>
+          <t>115370130</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>廖浚淇</t>
-        </is>
-      </c>
-      <c r="D113" t="inlineStr"/>
+          <t>易品妘</t>
+        </is>
+      </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>115370111</t>
+          <t>115370130</t>
         </is>
       </c>
     </row>
@@ -2966,18 +2954,17 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>115370112</t>
+          <t>115370131</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>吳亞叡</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr"/>
+          <t>張薇婷</t>
+        </is>
+      </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>115370112</t>
+          <t>115370131</t>
         </is>
       </c>
     </row>
@@ -2989,18 +2976,17 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>115370113</t>
+          <t>115370132</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>張洧豪</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr"/>
+          <t>蕭志杰</t>
+        </is>
+      </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>115370113</t>
+          <t>115370132</t>
         </is>
       </c>
     </row>
@@ -3012,18 +2998,17 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>115370114</t>
+          <t>115370133</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>陸捷</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr"/>
+          <t>彭榆真</t>
+        </is>
+      </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>115370114</t>
+          <t>115370133</t>
         </is>
       </c>
     </row>
@@ -3035,18 +3020,17 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>115370115</t>
+          <t>115370134</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>蔡幸恩</t>
-        </is>
-      </c>
-      <c r="D117" t="inlineStr"/>
+          <t>鄧妤溱</t>
+        </is>
+      </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>115370115</t>
+          <t>115370134</t>
         </is>
       </c>
     </row>
@@ -3058,18 +3042,17 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>115370116</t>
+          <t>115370135</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>康博閎</t>
-        </is>
-      </c>
-      <c r="D118" t="inlineStr"/>
+          <t>蔡其叡</t>
+        </is>
+      </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>115370116</t>
+          <t>115370135</t>
         </is>
       </c>
     </row>
@@ -3081,18 +3064,17 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>115370117</t>
+          <t>115370136</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>莫家葳</t>
-        </is>
-      </c>
-      <c r="D119" t="inlineStr"/>
+          <t>翁翊宸</t>
+        </is>
+      </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>115370117</t>
+          <t>115370136</t>
         </is>
       </c>
     </row>
@@ -3104,18 +3086,17 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>115370118</t>
+          <t>115370137</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>王義翔</t>
-        </is>
-      </c>
-      <c r="D120" t="inlineStr"/>
+          <t>陳柏霖</t>
+        </is>
+      </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>115370118</t>
+          <t>115370137</t>
         </is>
       </c>
     </row>
@@ -3127,18 +3108,17 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>115370119</t>
+          <t>115370138</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>譚佑捷</t>
-        </is>
-      </c>
-      <c r="D121" t="inlineStr"/>
+          <t>蔡侑霖</t>
+        </is>
+      </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>115370119</t>
+          <t>115370138</t>
         </is>
       </c>
     </row>
@@ -3150,18 +3130,17 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>115370120</t>
+          <t>115370139</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>林子佑</t>
-        </is>
-      </c>
-      <c r="D122" t="inlineStr"/>
+          <t>許凡羿</t>
+        </is>
+      </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>115370120</t>
+          <t>115370139</t>
         </is>
       </c>
     </row>
@@ -3173,18 +3152,17 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>115370121</t>
+          <t>115370140</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>陳右珊</t>
-        </is>
-      </c>
-      <c r="D123" t="inlineStr"/>
+          <t>宋世瑞</t>
+        </is>
+      </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>115370121</t>
+          <t>115370140</t>
         </is>
       </c>
     </row>
@@ -3196,18 +3174,17 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>115370122</t>
+          <t>115370141</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>楊仁佑</t>
-        </is>
-      </c>
-      <c r="D124" t="inlineStr"/>
+          <t>張瑞晏</t>
+        </is>
+      </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>115370122</t>
+          <t>115370141</t>
         </is>
       </c>
     </row>
@@ -3219,18 +3196,17 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>115370123</t>
+          <t>115370142</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>林洋宇</t>
-        </is>
-      </c>
-      <c r="D125" t="inlineStr"/>
+          <t>賴妍馨</t>
+        </is>
+      </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>115370123</t>
+          <t>115370142</t>
         </is>
       </c>
     </row>
@@ -3242,18 +3218,17 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>115370124</t>
+          <t>115370143</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>蔡承諺</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr"/>
+          <t>馮志恭</t>
+        </is>
+      </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>115370124</t>
+          <t>115370143</t>
         </is>
       </c>
     </row>
@@ -3265,18 +3240,17 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>115370125</t>
+          <t>115370144</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>蘇振綸</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr"/>
+          <t>謝玉玄</t>
+        </is>
+      </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>115370125</t>
+          <t>115370144</t>
         </is>
       </c>
     </row>
@@ -3288,18 +3262,17 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>115370126</t>
+          <t>115370145</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>陳億承</t>
-        </is>
-      </c>
-      <c r="D128" t="inlineStr"/>
+          <t>曾千財</t>
+        </is>
+      </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>115370126</t>
+          <t>115370145</t>
         </is>
       </c>
     </row>
@@ -3311,18 +3284,17 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>115370127</t>
+          <t>115370146</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>沈奕瑱</t>
-        </is>
-      </c>
-      <c r="D129" t="inlineStr"/>
+          <t>歐水愛</t>
+        </is>
+      </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>115370127</t>
+          <t>115370146</t>
         </is>
       </c>
     </row>
@@ -3334,18 +3306,17 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>115370128</t>
+          <t>115370147</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>翁敏瑄</t>
-        </is>
-      </c>
-      <c r="D130" t="inlineStr"/>
+          <t>思益邦</t>
+        </is>
+      </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>115370128</t>
+          <t>115370147</t>
         </is>
       </c>
     </row>
@@ -3357,18 +3328,17 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>115370129</t>
+          <t>115370148</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>傅可喬</t>
-        </is>
-      </c>
-      <c r="D131" t="inlineStr"/>
+          <t>楊詠訊</t>
+        </is>
+      </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>115370129</t>
+          <t>115370148</t>
         </is>
       </c>
     </row>
@@ -3380,18 +3350,17 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>115370130</t>
+          <t>112370116</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>易品妘</t>
-        </is>
-      </c>
-      <c r="D132" t="inlineStr"/>
+          <t>吳冠谷</t>
+        </is>
+      </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>115370130</t>
+          <t>112370116</t>
         </is>
       </c>
     </row>
@@ -3403,18 +3372,17 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>115370131</t>
+          <t>112370138</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>張薇婷</t>
-        </is>
-      </c>
-      <c r="D133" t="inlineStr"/>
+          <t>施皓偉</t>
+        </is>
+      </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>115370131</t>
+          <t>112370138</t>
         </is>
       </c>
     </row>
@@ -3426,18 +3394,17 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>115370132</t>
+          <t>112370140</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>蕭志杰</t>
-        </is>
-      </c>
-      <c r="D134" t="inlineStr"/>
+          <t>施廷儒</t>
+        </is>
+      </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>115370132</t>
+          <t>112370140</t>
         </is>
       </c>
     </row>
@@ -3449,453 +3416,15 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>115370133</t>
+          <t>112540024</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>彭榆真</t>
-        </is>
-      </c>
-      <c r="D135" t="inlineStr"/>
+          <t>廖芷葶</t>
+        </is>
+      </c>
       <c r="E135" t="inlineStr">
-        <is>
-          <t>115370133</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="inlineStr">
-        <is>
-          <t>course6</t>
-        </is>
-      </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>115370134</t>
-        </is>
-      </c>
-      <c r="C136" t="inlineStr">
-        <is>
-          <t>鄧妤溱</t>
-        </is>
-      </c>
-      <c r="D136" t="inlineStr"/>
-      <c r="E136" t="inlineStr">
-        <is>
-          <t>115370134</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" t="inlineStr">
-        <is>
-          <t>course6</t>
-        </is>
-      </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>115370135</t>
-        </is>
-      </c>
-      <c r="C137" t="inlineStr">
-        <is>
-          <t>蔡其叡</t>
-        </is>
-      </c>
-      <c r="D137" t="inlineStr"/>
-      <c r="E137" t="inlineStr">
-        <is>
-          <t>115370135</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" t="inlineStr">
-        <is>
-          <t>course6</t>
-        </is>
-      </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>115370136</t>
-        </is>
-      </c>
-      <c r="C138" t="inlineStr">
-        <is>
-          <t>翁翊宸</t>
-        </is>
-      </c>
-      <c r="D138" t="inlineStr"/>
-      <c r="E138" t="inlineStr">
-        <is>
-          <t>115370136</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" t="inlineStr">
-        <is>
-          <t>course6</t>
-        </is>
-      </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>115370137</t>
-        </is>
-      </c>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>陳柏霖</t>
-        </is>
-      </c>
-      <c r="D139" t="inlineStr"/>
-      <c r="E139" t="inlineStr">
-        <is>
-          <t>115370137</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="inlineStr">
-        <is>
-          <t>course6</t>
-        </is>
-      </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>115370138</t>
-        </is>
-      </c>
-      <c r="C140" t="inlineStr">
-        <is>
-          <t>蔡侑霖</t>
-        </is>
-      </c>
-      <c r="D140" t="inlineStr"/>
-      <c r="E140" t="inlineStr">
-        <is>
-          <t>115370138</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" t="inlineStr">
-        <is>
-          <t>course6</t>
-        </is>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>115370139</t>
-        </is>
-      </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>許凡羿</t>
-        </is>
-      </c>
-      <c r="D141" t="inlineStr"/>
-      <c r="E141" t="inlineStr">
-        <is>
-          <t>115370139</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t>course6</t>
-        </is>
-      </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>115370140</t>
-        </is>
-      </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t>宋世瑞</t>
-        </is>
-      </c>
-      <c r="D142" t="inlineStr"/>
-      <c r="E142" t="inlineStr">
-        <is>
-          <t>115370140</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" t="inlineStr">
-        <is>
-          <t>course6</t>
-        </is>
-      </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>115370141</t>
-        </is>
-      </c>
-      <c r="C143" t="inlineStr">
-        <is>
-          <t>張瑞晏</t>
-        </is>
-      </c>
-      <c r="D143" t="inlineStr"/>
-      <c r="E143" t="inlineStr">
-        <is>
-          <t>115370141</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" t="inlineStr">
-        <is>
-          <t>course6</t>
-        </is>
-      </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>115370142</t>
-        </is>
-      </c>
-      <c r="C144" t="inlineStr">
-        <is>
-          <t>賴妍馨</t>
-        </is>
-      </c>
-      <c r="D144" t="inlineStr"/>
-      <c r="E144" t="inlineStr">
-        <is>
-          <t>115370142</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" t="inlineStr">
-        <is>
-          <t>course6</t>
-        </is>
-      </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>115370143</t>
-        </is>
-      </c>
-      <c r="C145" t="inlineStr">
-        <is>
-          <t>馮志恭</t>
-        </is>
-      </c>
-      <c r="D145" t="inlineStr"/>
-      <c r="E145" t="inlineStr">
-        <is>
-          <t>115370143</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" t="inlineStr">
-        <is>
-          <t>course6</t>
-        </is>
-      </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>115370144</t>
-        </is>
-      </c>
-      <c r="C146" t="inlineStr">
-        <is>
-          <t>謝玉玄</t>
-        </is>
-      </c>
-      <c r="D146" t="inlineStr"/>
-      <c r="E146" t="inlineStr">
-        <is>
-          <t>115370144</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" t="inlineStr">
-        <is>
-          <t>course6</t>
-        </is>
-      </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>115370145</t>
-        </is>
-      </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>曾千財</t>
-        </is>
-      </c>
-      <c r="D147" t="inlineStr"/>
-      <c r="E147" t="inlineStr">
-        <is>
-          <t>115370145</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>course6</t>
-        </is>
-      </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>115370146</t>
-        </is>
-      </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>歐水愛</t>
-        </is>
-      </c>
-      <c r="D148" t="inlineStr"/>
-      <c r="E148" t="inlineStr">
-        <is>
-          <t>115370146</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>course6</t>
-        </is>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>115370147</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>思益邦</t>
-        </is>
-      </c>
-      <c r="D149" t="inlineStr"/>
-      <c r="E149" t="inlineStr">
-        <is>
-          <t>115370147</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>course6</t>
-        </is>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>115370148</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>楊詠訊</t>
-        </is>
-      </c>
-      <c r="D150" t="inlineStr"/>
-      <c r="E150" t="inlineStr">
-        <is>
-          <t>115370148</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t>course6</t>
-        </is>
-      </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>112370116</t>
-        </is>
-      </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>吳冠谷</t>
-        </is>
-      </c>
-      <c r="D151" t="inlineStr"/>
-      <c r="E151" t="inlineStr">
-        <is>
-          <t>112370116</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t>course6</t>
-        </is>
-      </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>112370138</t>
-        </is>
-      </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>施皓偉</t>
-        </is>
-      </c>
-      <c r="D152" t="inlineStr"/>
-      <c r="E152" t="inlineStr">
-        <is>
-          <t>112370138</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>course6</t>
-        </is>
-      </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>112370140</t>
-        </is>
-      </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>施廷儒</t>
-        </is>
-      </c>
-      <c r="D153" t="inlineStr"/>
-      <c r="E153" t="inlineStr">
-        <is>
-          <t>112370140</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="inlineStr">
-        <is>
-          <t>course6</t>
-        </is>
-      </c>
-      <c r="B154" t="inlineStr">
-        <is>
-          <t>112540024</t>
-        </is>
-      </c>
-      <c r="C154" t="inlineStr">
-        <is>
-          <t>廖芷葶</t>
-        </is>
-      </c>
-      <c r="D154" t="inlineStr"/>
-      <c r="E154" t="inlineStr">
         <is>
           <t>112540024</t>
         </is>

</xml_diff>

<commit_message>
feat: add Jessica to course5 roster
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/students.xlsx
+++ b/data/students.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D161"/>
+  <dimension ref="A1:D162"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2653,9 +2653,23 @@
         <v>115C26528</v>
       </c>
     </row>
+    <row r="162">
+      <c r="A162" t="str">
+        <v>course5</v>
+      </c>
+      <c r="B162" t="str">
+        <v>Jessica</v>
+      </c>
+      <c r="C162" t="str">
+        <v>Jessica</v>
+      </c>
+      <c r="D162" t="str">
+        <v>Jessica</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D161"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D162"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>